<commit_message>
feat(transactions): add event_timestamp column migration and decouple synthetic fixture identities
</commit_message>
<xml_diff>
--- a/backend/app/data/v14_temporal_fixture.xlsx
+++ b/backend/app/data/v14_temporal_fixture.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,20 +575,25 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>event_timestamp</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>approval_required</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>approval_status</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>payment_status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -628,20 +633,25 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="H2" t="b">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-08-28 10:14:00</t>
+        </is>
+      </c>
+      <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Material infrastructure payment (TX-TEMP-001)</t>
         </is>
@@ -1020,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1036,25 +1046,30 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>primary_record</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>expected_priority</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>assigned_to</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -1073,25 +1088,30 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>TX-TEMP-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>SUP-TEMP-001</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>usr-reviewer-01</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Temporal surveillance case for TX-TEMP-001</t>
         </is>

</xml_diff>